<commit_message>
Taco voador do Maues (BUILD 202610211420)
Co-authored-by: matmaues <matmaues@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kit/personagens.xlsx
+++ b/kit/personagens.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>chinelo</t>
+          <t>taco</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>CHINELADA</t>
+          <t>TACO VOADOR</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>SUPER CHINELADA</t>
+          <t>SUPER TACADA</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">

</xml_diff>

<commit_message>
Milk, Clube Chalezinho, frases (BUILD 202610211440)
Co-authored-by: matmaues <matmaues@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kit/personagens.xlsx
+++ b/kit/personagens.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMO USAR" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especiais" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Golpes básicos (ref.)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frases" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Golpes básicos (ref.)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -486,50 +487,57 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Frases de vitória: aba Frases (uma por linha; o jogo sorteia uma).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>5. Troque o número BUILD no index.html e publique. Pronto!</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Dicas de balanceamento:</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>- Velocidade, Força e Vida vão de 1 a 10. Vida real = 60 + Vida × 8. Dano real = dano base × (0,6 + Força × 0,09).</t>
+          <t>Dicas de balanceamento:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- Personagens devem ser DIFERENTES (ex.: rápido e fraco x lento e forte). Mire em 45–55% de vitórias:</t>
+          <t>- Velocidade, Força e Vida vão de 1 a 10. Vida real = 60 + Vida × 8. Dano real = dano base × (0,6 + Força × 0,09).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  node tools/sim.js '&lt;stats&gt;' 200  (com o servidor local ligado) mede isso.</t>
+          <t>- Personagens devem ser DIFERENTES (ex.: rápido e fraco x lento e forte). Mire em 45–55% de vitórias:</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>- Frames: 60 frames = 1 segundo. Início menor = golpe sai mais rápido. Recuperação maior = mais fácil de punir.</t>
+          <t xml:space="preserve">  node tools/sim.js '&lt;stats&gt;' 200  (com o servidor local ligado) mede isso.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>- Frames: 60 frames = 1 segundo. Início menor = golpe sai mais rápido. Recuperação maior = mais fácil de punir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>- Para voltar tudo ao padrão: python3 tools/planilha.py exportar (recria a planilha a partir do jogo).</t>
         </is>
@@ -546,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -559,7 +567,6 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -613,11 +620,6 @@
           <t>Projétil (desenho)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Frase de vitória</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -660,11 +662,6 @@
           <t>taco</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Chinelo branco não perdoa ninguém!</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -707,24 +704,21 @@
           <t>granada</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Missão cumprida. Próximo da fila!</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lutador 3</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n"/>
+          <t>Milk</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1.78</v>
+      </c>
       <c r="C4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>8</v>
@@ -739,36 +733,35 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>#3bd16f</t>
+          <t>#5b3fa0</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>#1a1a1a</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Força bruta resolve tudo.</t>
+          <t>#f4f4ff</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>pituxo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lutador 4</t>
+          <t>Lutador 3</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F5">
         <f>60+E5*8</f>
@@ -780,25 +773,20 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>#b03be8</t>
+          <t>#3bd16f</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>#ff9ff3</t>
+          <t>#1a1a1a</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Volte quando treinar mais.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chefão</t>
+          <t>Lutador 4</t>
         </is>
       </c>
       <c r="B6" s="3" t="n"/>
@@ -806,10 +794,10 @@
         <v>7</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F6">
         <f>60+E6*8</f>
@@ -821,24 +809,55 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>#b03be8</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>#ff9ff3</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Chefão</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7">
+        <f>60+E7*8</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>C7+D7+E7</f>
+        <v/>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
           <t>#2b2b33</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>#e83b3b</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Ninguém derruba o Chefão!</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:E2 C3:E3 C4:E4 C5:E5 C6:E6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Use um número de 1 a 10" type="whole" operator="between">
+    <dataValidation sqref="C2:E2 C3:E3 C4:E4 C5:E5 C6:E6 C7:E7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Use um número de 1 a 10" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -853,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1281,7 +1300,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lutador 3</t>
+          <t>Milk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1296,7 +1315,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>PEDRADA</t>
+          <t>PITUXO</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -1326,7 +1345,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lutador 3</t>
+          <t>Milk</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1341,7 +1360,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>GANCHO DE PEDRA</t>
+          <t>GANCHO DO MILK</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -1369,7 +1388,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Lutador 3</t>
+          <t>Milk</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1384,7 +1403,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>ROLO COMPRESSOR</t>
+          <t>BARRIGADA GIRATÓRIA</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -1412,7 +1431,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Lutador 3</t>
+          <t>Milk</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1427,7 +1446,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>TERREMOTO TOTAL</t>
+          <t>SUPER PITUXO</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -1457,7 +1476,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Lutador 4</t>
+          <t>Lutador 3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1472,7 +1491,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>RAIO ROXO</t>
+          <t>PEDRADA</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
@@ -1502,7 +1521,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lutador 4</t>
+          <t>Lutador 3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1517,7 +1536,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>GANCHO VOADOR</t>
+          <t>GANCHO DE PEDRA</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
@@ -1545,7 +1564,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lutador 4</t>
+          <t>Lutador 3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1560,7 +1579,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>PIÃO ROXO</t>
+          <t>ROLO COMPRESSOR</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -1588,7 +1607,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lutador 4</t>
+          <t>Lutador 3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1603,7 +1622,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>FÚRIA VIOLETA</t>
+          <t>TERREMOTO TOTAL</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
@@ -1633,7 +1652,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Chefão</t>
+          <t>Lutador 4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1648,7 +1667,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>BOLA SOMBRIA</t>
+          <t>RAIO ROXO</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
@@ -1678,7 +1697,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Chefão</t>
+          <t>Lutador 4</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1693,7 +1712,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>GANCHO DO CHEFÃO</t>
+          <t>GANCHO VOADOR</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
@@ -1721,7 +1740,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Chefão</t>
+          <t>Lutador 4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1736,7 +1755,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>FURACÃO SOMBRIO</t>
+          <t>PIÃO ROXO</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
@@ -1764,7 +1783,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Chefão</t>
+          <t>Lutador 4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1779,7 +1798,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>APOCALIPSE</t>
+          <t>FÚRIA VIOLETA</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
@@ -1801,6 +1820,182 @@
         <v>5</v>
       </c>
       <c r="K21" t="inlineStr">
+        <is>
+          <t>super</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Chefão</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Projétil</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>↓ ↘ → + soco</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>BOLA SOMBRIA</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>fireball</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Chefão</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gancho anti-aéreo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>→ ↓ ↘ + soco</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>GANCHO DO CHEFÃO</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>dp</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Chefão</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Furacão</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>↓ ↙ ← + chute</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>FURACÃO SOMBRIO</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>spin</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Chefão</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Super</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>↓↘→ ↓↘→ + soco (barra cheia)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>APOCALIPSE</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>super</t>
         </is>
@@ -1812,6 +2007,139 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Frase de vitória (uma por linha; o jogo sorteia uma)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Maués</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Chinelo branco não perdoa ninguém!</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>João Pedro</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Missão cumprida. Próximo da fila!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Milk</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Toma leite que passa!</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Milk</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Um Pituxo pra comemorar!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Milk</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Barriga de respeito, golpe de respeito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lutador 3</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Força bruta resolve tudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lutador 4</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Volte quando treinar mais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Chefão</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Ninguém derruba o Chefão!</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>(para adicionar uma frase, insira uma linha com o Nome do personagem e a frase)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Cotovelos Joao/Milk, frase Milk (BUILD 202610211500)
Co-authored-by: matmaues <matmaues@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kit/personagens.xlsx
+++ b/kit/personagens.xlsx
@@ -2012,7 +2012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2063,72 +2063,48 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Toma leite que passa!</t>
+          <t>Pix sem taxa no pv</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Milk</t>
+          <t>Lutador 3</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Um Pituxo pra comemorar!</t>
+          <t>Força bruta resolve tudo.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Milk</t>
+          <t>Lutador 4</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Barriga de respeito, golpe de respeito.</t>
+          <t>Volte quando treinar mais.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lutador 3</t>
+          <t>Chefão</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Força bruta resolve tudo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Lutador 4</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Volte quando treinar mais.</t>
+          <t>Ninguém derruba o Chefão!</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
-        <is>
-          <t>Chefão</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Ninguém derruba o Chefão!</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
         <is>
           <t>(para adicionar uma frase, insira uma linha com o Nome do personagem e a frase)</t>
         </is>

</xml_diff>